<commit_message>
로봇 자동 갱신: 2026-10-12
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11205" uniqueCount="5556">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11209" uniqueCount="5558">
   <si>
     <t>연번</t>
   </si>
@@ -1052,12 +1052,12 @@
     <t>사루</t>
   </si>
   <si>
+    <t>서울특별시 중구 동호로12길 53(1층 신당동)</t>
+  </si>
+  <si>
     <t>서울특별시 중구 장충단로7길 24(1층 쌍림동)</t>
   </si>
   <si>
-    <t>서울특별시 중구 동호로12길 53(1층 신당동)</t>
-  </si>
-  <si>
     <t>사직커피</t>
   </si>
   <si>
@@ -1541,12 +1541,12 @@
     <t>오르노 합정점</t>
   </si>
   <si>
+    <t>서울특별시 마포구 월드컵로3길 14(지1층 B113,114호 합정동, 마포 한강 2차 푸르지오)</t>
+  </si>
+  <si>
     <t>서울특별시 마포구 월드컵로3길 14(지1층 B149,B150,B151, B152,B153,B154호 합정동, 마포 한강 2차 푸르지오)</t>
   </si>
   <si>
-    <t>서울특별시 마포구 월드컵로3길 14(지1층 B113,114호 합정동, 마포 한강 2차 푸르지오)</t>
-  </si>
-  <si>
     <t>오베뉴 한남</t>
   </si>
   <si>
@@ -5996,12 +5996,12 @@
     <t>조선백호</t>
   </si>
   <si>
+    <t>인천광역시 제물포구 개항로96번길 11(1,2층 경동)</t>
+  </si>
+  <si>
     <t>인천광역시 제물포구 개항로96번길 11(1층 경동)</t>
   </si>
   <si>
-    <t>인천광역시 제물포구 개항로96번길 11(1,2층 경동)</t>
-  </si>
-  <si>
     <t>주윤 상차림</t>
   </si>
   <si>
@@ -6215,12 +6215,12 @@
     <t>그리너리 바스켓</t>
   </si>
   <si>
+    <t>인천광역시 영종구 백운로 510(1동 지1층 운북동)</t>
+  </si>
+  <si>
     <t>인천광역시 영종구 백운로 510(2동 1,2층 운북동)</t>
   </si>
   <si>
-    <t>인천광역시 영종구 백운로 510(1동 지1층 운북동)</t>
-  </si>
-  <si>
     <t>까페마인</t>
   </si>
   <si>
@@ -14712,6 +14712,12 @@
   </si>
   <si>
     <t>제주특별자치도 제주시 서부두길 22(1~3층 제4호 건입동)</t>
+  </si>
+  <si>
+    <t>오늘이크리스마스라면 사진관카페</t>
+  </si>
+  <si>
+    <t>제주특별자치도 서귀포시 성산읍 일주동로5154번길 5(1층)</t>
   </si>
   <si>
     <t>오롬마르</t>
@@ -59084,7 +59090,7 @@
         <v>4938</v>
       </c>
       <c r="C2489" t="s" s="2">
-        <v>792</v>
+        <v>6</v>
       </c>
       <c r="D2489" t="s" s="2">
         <v>4828</v>
@@ -59730,7 +59736,7 @@
         <v>5014</v>
       </c>
       <c r="C2527" t="s" s="2">
-        <v>1011</v>
+        <v>792</v>
       </c>
       <c r="D2527" t="s" s="2">
         <v>4828</v>
@@ -59866,13 +59872,13 @@
         <v>5030</v>
       </c>
       <c r="C2535" t="s" s="2">
-        <v>6</v>
+        <v>1011</v>
       </c>
       <c r="D2535" t="s" s="2">
+        <v>4828</v>
+      </c>
+      <c r="E2535" t="s" s="3">
         <v>5031</v>
-      </c>
-      <c r="E2535" t="s" s="3">
-        <v>5032</v>
       </c>
     </row>
     <row r="2536" ht="36.0" customHeight="true">
@@ -59880,13 +59886,13 @@
         <v>2535.0</v>
       </c>
       <c r="B2536" t="s" s="3">
+        <v>5032</v>
+      </c>
+      <c r="C2536" t="s" s="2">
+        <v>6</v>
+      </c>
+      <c r="D2536" t="s" s="2">
         <v>5033</v>
-      </c>
-      <c r="C2536" t="s" s="2">
-        <v>6</v>
-      </c>
-      <c r="D2536" t="s" s="2">
-        <v>5031</v>
       </c>
       <c r="E2536" t="s" s="3">
         <v>5034</v>
@@ -59903,7 +59909,7 @@
         <v>6</v>
       </c>
       <c r="D2537" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2537" t="s" s="3">
         <v>5036</v>
@@ -59920,7 +59926,7 @@
         <v>6</v>
       </c>
       <c r="D2538" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2538" t="s" s="3">
         <v>5038</v>
@@ -59937,7 +59943,7 @@
         <v>6</v>
       </c>
       <c r="D2539" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2539" t="s" s="3">
         <v>5040</v>
@@ -59954,7 +59960,7 @@
         <v>6</v>
       </c>
       <c r="D2540" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2540" t="s" s="3">
         <v>5042</v>
@@ -59971,7 +59977,7 @@
         <v>6</v>
       </c>
       <c r="D2541" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2541" t="s" s="3">
         <v>5044</v>
@@ -59988,7 +59994,7 @@
         <v>6</v>
       </c>
       <c r="D2542" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2542" t="s" s="3">
         <v>5046</v>
@@ -60005,7 +60011,7 @@
         <v>6</v>
       </c>
       <c r="D2543" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2543" t="s" s="3">
         <v>5048</v>
@@ -60022,7 +60028,7 @@
         <v>6</v>
       </c>
       <c r="D2544" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2544" t="s" s="3">
         <v>5050</v>
@@ -60039,7 +60045,7 @@
         <v>6</v>
       </c>
       <c r="D2545" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2545" t="s" s="3">
         <v>5052</v>
@@ -60056,7 +60062,7 @@
         <v>6</v>
       </c>
       <c r="D2546" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2546" t="s" s="3">
         <v>5054</v>
@@ -60073,7 +60079,7 @@
         <v>6</v>
       </c>
       <c r="D2547" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2547" t="s" s="3">
         <v>5056</v>
@@ -60090,7 +60096,7 @@
         <v>6</v>
       </c>
       <c r="D2548" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2548" t="s" s="3">
         <v>5058</v>
@@ -60107,7 +60113,7 @@
         <v>6</v>
       </c>
       <c r="D2549" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2549" t="s" s="3">
         <v>5060</v>
@@ -60124,7 +60130,7 @@
         <v>6</v>
       </c>
       <c r="D2550" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2550" t="s" s="3">
         <v>5062</v>
@@ -60141,7 +60147,7 @@
         <v>6</v>
       </c>
       <c r="D2551" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2551" t="s" s="3">
         <v>5064</v>
@@ -60158,7 +60164,7 @@
         <v>6</v>
       </c>
       <c r="D2552" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2552" t="s" s="3">
         <v>5066</v>
@@ -60175,7 +60181,7 @@
         <v>6</v>
       </c>
       <c r="D2553" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2553" t="s" s="3">
         <v>5068</v>
@@ -60192,7 +60198,7 @@
         <v>6</v>
       </c>
       <c r="D2554" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2554" t="s" s="3">
         <v>5070</v>
@@ -60209,7 +60215,7 @@
         <v>6</v>
       </c>
       <c r="D2555" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2555" t="s" s="3">
         <v>5072</v>
@@ -60226,7 +60232,7 @@
         <v>6</v>
       </c>
       <c r="D2556" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2556" t="s" s="3">
         <v>5074</v>
@@ -60243,7 +60249,7 @@
         <v>6</v>
       </c>
       <c r="D2557" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2557" t="s" s="3">
         <v>5076</v>
@@ -60260,7 +60266,7 @@
         <v>6</v>
       </c>
       <c r="D2558" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2558" t="s" s="3">
         <v>5078</v>
@@ -60277,7 +60283,7 @@
         <v>6</v>
       </c>
       <c r="D2559" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2559" t="s" s="3">
         <v>5080</v>
@@ -60294,7 +60300,7 @@
         <v>6</v>
       </c>
       <c r="D2560" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2560" t="s" s="3">
         <v>5082</v>
@@ -60311,7 +60317,7 @@
         <v>6</v>
       </c>
       <c r="D2561" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2561" t="s" s="3">
         <v>5084</v>
@@ -60328,7 +60334,7 @@
         <v>6</v>
       </c>
       <c r="D2562" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2562" t="s" s="3">
         <v>5086</v>
@@ -60345,7 +60351,7 @@
         <v>6</v>
       </c>
       <c r="D2563" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2563" t="s" s="3">
         <v>5088</v>
@@ -60362,7 +60368,7 @@
         <v>6</v>
       </c>
       <c r="D2564" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2564" t="s" s="3">
         <v>5090</v>
@@ -60379,7 +60385,7 @@
         <v>6</v>
       </c>
       <c r="D2565" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2565" t="s" s="3">
         <v>5092</v>
@@ -60396,7 +60402,7 @@
         <v>6</v>
       </c>
       <c r="D2566" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2566" t="s" s="3">
         <v>5094</v>
@@ -60413,7 +60419,7 @@
         <v>6</v>
       </c>
       <c r="D2567" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2567" t="s" s="3">
         <v>5096</v>
@@ -60430,7 +60436,7 @@
         <v>6</v>
       </c>
       <c r="D2568" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2568" t="s" s="3">
         <v>5098</v>
@@ -60447,7 +60453,7 @@
         <v>6</v>
       </c>
       <c r="D2569" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2569" t="s" s="3">
         <v>5100</v>
@@ -60464,7 +60470,7 @@
         <v>6</v>
       </c>
       <c r="D2570" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2570" t="s" s="3">
         <v>5102</v>
@@ -60481,7 +60487,7 @@
         <v>6</v>
       </c>
       <c r="D2571" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2571" t="s" s="3">
         <v>5104</v>
@@ -60498,7 +60504,7 @@
         <v>6</v>
       </c>
       <c r="D2572" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2572" t="s" s="3">
         <v>5106</v>
@@ -60515,7 +60521,7 @@
         <v>6</v>
       </c>
       <c r="D2573" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2573" t="s" s="3">
         <v>5108</v>
@@ -60532,7 +60538,7 @@
         <v>6</v>
       </c>
       <c r="D2574" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2574" t="s" s="3">
         <v>5110</v>
@@ -60549,7 +60555,7 @@
         <v>6</v>
       </c>
       <c r="D2575" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2575" t="s" s="3">
         <v>5112</v>
@@ -60566,7 +60572,7 @@
         <v>6</v>
       </c>
       <c r="D2576" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2576" t="s" s="3">
         <v>5114</v>
@@ -60583,7 +60589,7 @@
         <v>6</v>
       </c>
       <c r="D2577" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2577" t="s" s="3">
         <v>5116</v>
@@ -60600,7 +60606,7 @@
         <v>6</v>
       </c>
       <c r="D2578" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2578" t="s" s="3">
         <v>5118</v>
@@ -60617,7 +60623,7 @@
         <v>6</v>
       </c>
       <c r="D2579" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2579" t="s" s="3">
         <v>5120</v>
@@ -60634,7 +60640,7 @@
         <v>6</v>
       </c>
       <c r="D2580" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2580" t="s" s="3">
         <v>5122</v>
@@ -60651,7 +60657,7 @@
         <v>6</v>
       </c>
       <c r="D2581" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2581" t="s" s="3">
         <v>5124</v>
@@ -60668,7 +60674,7 @@
         <v>6</v>
       </c>
       <c r="D2582" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2582" t="s" s="3">
         <v>5126</v>
@@ -60685,7 +60691,7 @@
         <v>6</v>
       </c>
       <c r="D2583" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2583" t="s" s="3">
         <v>5128</v>
@@ -60702,7 +60708,7 @@
         <v>6</v>
       </c>
       <c r="D2584" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2584" t="s" s="3">
         <v>5130</v>
@@ -60719,7 +60725,7 @@
         <v>6</v>
       </c>
       <c r="D2585" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2585" t="s" s="3">
         <v>5132</v>
@@ -60736,7 +60742,7 @@
         <v>6</v>
       </c>
       <c r="D2586" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2586" t="s" s="3">
         <v>5134</v>
@@ -60753,7 +60759,7 @@
         <v>6</v>
       </c>
       <c r="D2587" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2587" t="s" s="3">
         <v>5136</v>
@@ -60770,7 +60776,7 @@
         <v>6</v>
       </c>
       <c r="D2588" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2588" t="s" s="3">
         <v>5138</v>
@@ -60787,7 +60793,7 @@
         <v>6</v>
       </c>
       <c r="D2589" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2589" t="s" s="3">
         <v>5140</v>
@@ -60804,7 +60810,7 @@
         <v>6</v>
       </c>
       <c r="D2590" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2590" t="s" s="3">
         <v>5142</v>
@@ -60821,7 +60827,7 @@
         <v>6</v>
       </c>
       <c r="D2591" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2591" t="s" s="3">
         <v>5144</v>
@@ -60838,7 +60844,7 @@
         <v>6</v>
       </c>
       <c r="D2592" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2592" t="s" s="3">
         <v>5146</v>
@@ -60855,7 +60861,7 @@
         <v>6</v>
       </c>
       <c r="D2593" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2593" t="s" s="3">
         <v>5148</v>
@@ -60872,7 +60878,7 @@
         <v>6</v>
       </c>
       <c r="D2594" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2594" t="s" s="3">
         <v>5150</v>
@@ -60889,7 +60895,7 @@
         <v>6</v>
       </c>
       <c r="D2595" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2595" t="s" s="3">
         <v>5152</v>
@@ -60906,7 +60912,7 @@
         <v>6</v>
       </c>
       <c r="D2596" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2596" t="s" s="3">
         <v>5154</v>
@@ -60923,7 +60929,7 @@
         <v>6</v>
       </c>
       <c r="D2597" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2597" t="s" s="3">
         <v>5156</v>
@@ -60940,7 +60946,7 @@
         <v>6</v>
       </c>
       <c r="D2598" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2598" t="s" s="3">
         <v>5158</v>
@@ -60957,7 +60963,7 @@
         <v>6</v>
       </c>
       <c r="D2599" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2599" t="s" s="3">
         <v>5160</v>
@@ -60974,7 +60980,7 @@
         <v>6</v>
       </c>
       <c r="D2600" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2600" t="s" s="3">
         <v>5162</v>
@@ -60991,7 +60997,7 @@
         <v>6</v>
       </c>
       <c r="D2601" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2601" t="s" s="3">
         <v>5164</v>
@@ -61008,7 +61014,7 @@
         <v>6</v>
       </c>
       <c r="D2602" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2602" t="s" s="3">
         <v>5166</v>
@@ -61025,7 +61031,7 @@
         <v>6</v>
       </c>
       <c r="D2603" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2603" t="s" s="3">
         <v>5168</v>
@@ -61042,7 +61048,7 @@
         <v>6</v>
       </c>
       <c r="D2604" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2604" t="s" s="3">
         <v>5170</v>
@@ -61059,7 +61065,7 @@
         <v>6</v>
       </c>
       <c r="D2605" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2605" t="s" s="3">
         <v>5172</v>
@@ -61076,7 +61082,7 @@
         <v>6</v>
       </c>
       <c r="D2606" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2606" t="s" s="3">
         <v>5174</v>
@@ -61093,7 +61099,7 @@
         <v>6</v>
       </c>
       <c r="D2607" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2607" t="s" s="3">
         <v>5176</v>
@@ -61110,7 +61116,7 @@
         <v>6</v>
       </c>
       <c r="D2608" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2608" t="s" s="3">
         <v>5178</v>
@@ -61127,10 +61133,10 @@
         <v>6</v>
       </c>
       <c r="D2609" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2609" t="s" s="3">
-        <v>5148</v>
+        <v>5180</v>
       </c>
     </row>
     <row r="2610" ht="36.0" customHeight="true">
@@ -61138,16 +61144,16 @@
         <v>2609.0</v>
       </c>
       <c r="B2610" t="s" s="3">
-        <v>5180</v>
+        <v>5181</v>
       </c>
       <c r="C2610" t="s" s="2">
         <v>6</v>
       </c>
       <c r="D2610" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2610" t="s" s="3">
-        <v>5181</v>
+        <v>5150</v>
       </c>
     </row>
     <row r="2611" ht="36.0" customHeight="true">
@@ -61161,7 +61167,7 @@
         <v>6</v>
       </c>
       <c r="D2611" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2611" t="s" s="3">
         <v>5183</v>
@@ -61178,7 +61184,7 @@
         <v>6</v>
       </c>
       <c r="D2612" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2612" t="s" s="3">
         <v>5185</v>
@@ -61195,7 +61201,7 @@
         <v>6</v>
       </c>
       <c r="D2613" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2613" t="s" s="3">
         <v>5187</v>
@@ -61212,7 +61218,7 @@
         <v>6</v>
       </c>
       <c r="D2614" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2614" t="s" s="3">
         <v>5189</v>
@@ -61229,7 +61235,7 @@
         <v>6</v>
       </c>
       <c r="D2615" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2615" t="s" s="3">
         <v>5191</v>
@@ -61246,7 +61252,7 @@
         <v>6</v>
       </c>
       <c r="D2616" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2616" t="s" s="3">
         <v>5193</v>
@@ -61263,10 +61269,10 @@
         <v>6</v>
       </c>
       <c r="D2617" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2617" t="s" s="3">
-        <v>5110</v>
+        <v>5195</v>
       </c>
     </row>
     <row r="2618" ht="36.0" customHeight="true">
@@ -61274,16 +61280,16 @@
         <v>2617.0</v>
       </c>
       <c r="B2618" t="s" s="3">
-        <v>4180</v>
+        <v>5196</v>
       </c>
       <c r="C2618" t="s" s="2">
         <v>6</v>
       </c>
       <c r="D2618" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2618" t="s" s="3">
-        <v>5195</v>
+        <v>5112</v>
       </c>
     </row>
     <row r="2619" ht="36.0" customHeight="true">
@@ -61291,16 +61297,16 @@
         <v>2618.0</v>
       </c>
       <c r="B2619" t="s" s="3">
-        <v>5196</v>
+        <v>4180</v>
       </c>
       <c r="C2619" t="s" s="2">
         <v>6</v>
       </c>
       <c r="D2619" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2619" t="s" s="3">
-        <v>5148</v>
+        <v>5197</v>
       </c>
     </row>
     <row r="2620" ht="36.0" customHeight="true">
@@ -61308,16 +61314,16 @@
         <v>2619.0</v>
       </c>
       <c r="B2620" t="s" s="3">
-        <v>5197</v>
+        <v>5198</v>
       </c>
       <c r="C2620" t="s" s="2">
         <v>6</v>
       </c>
       <c r="D2620" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2620" t="s" s="3">
-        <v>5198</v>
+        <v>5150</v>
       </c>
     </row>
     <row r="2621" ht="36.0" customHeight="true">
@@ -61331,7 +61337,7 @@
         <v>6</v>
       </c>
       <c r="D2621" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2621" t="s" s="3">
         <v>5200</v>
@@ -61348,7 +61354,7 @@
         <v>6</v>
       </c>
       <c r="D2622" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2622" t="s" s="3">
         <v>5202</v>
@@ -61365,7 +61371,7 @@
         <v>6</v>
       </c>
       <c r="D2623" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2623" t="s" s="3">
         <v>5204</v>
@@ -61382,7 +61388,7 @@
         <v>6</v>
       </c>
       <c r="D2624" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2624" t="s" s="3">
         <v>5206</v>
@@ -61399,7 +61405,7 @@
         <v>6</v>
       </c>
       <c r="D2625" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2625" t="s" s="3">
         <v>5208</v>
@@ -61416,7 +61422,7 @@
         <v>6</v>
       </c>
       <c r="D2626" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2626" t="s" s="3">
         <v>5210</v>
@@ -61433,7 +61439,7 @@
         <v>6</v>
       </c>
       <c r="D2627" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2627" t="s" s="3">
         <v>5212</v>
@@ -61450,7 +61456,7 @@
         <v>6</v>
       </c>
       <c r="D2628" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2628" t="s" s="3">
         <v>5214</v>
@@ -61467,7 +61473,7 @@
         <v>6</v>
       </c>
       <c r="D2629" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2629" t="s" s="3">
         <v>5216</v>
@@ -61484,7 +61490,7 @@
         <v>6</v>
       </c>
       <c r="D2630" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2630" t="s" s="3">
         <v>5218</v>
@@ -61501,7 +61507,7 @@
         <v>6</v>
       </c>
       <c r="D2631" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2631" t="s" s="3">
         <v>5220</v>
@@ -61518,7 +61524,7 @@
         <v>6</v>
       </c>
       <c r="D2632" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2632" t="s" s="3">
         <v>5222</v>
@@ -61535,7 +61541,7 @@
         <v>6</v>
       </c>
       <c r="D2633" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2633" t="s" s="3">
         <v>5224</v>
@@ -61552,7 +61558,7 @@
         <v>6</v>
       </c>
       <c r="D2634" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2634" t="s" s="3">
         <v>5226</v>
@@ -61569,7 +61575,7 @@
         <v>6</v>
       </c>
       <c r="D2635" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2635" t="s" s="3">
         <v>5228</v>
@@ -61586,7 +61592,7 @@
         <v>6</v>
       </c>
       <c r="D2636" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2636" t="s" s="3">
         <v>5230</v>
@@ -61603,7 +61609,7 @@
         <v>6</v>
       </c>
       <c r="D2637" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2637" t="s" s="3">
         <v>5232</v>
@@ -61620,7 +61626,7 @@
         <v>6</v>
       </c>
       <c r="D2638" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2638" t="s" s="3">
         <v>5234</v>
@@ -61637,7 +61643,7 @@
         <v>6</v>
       </c>
       <c r="D2639" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2639" t="s" s="3">
         <v>5236</v>
@@ -61654,7 +61660,7 @@
         <v>6</v>
       </c>
       <c r="D2640" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2640" t="s" s="3">
         <v>5238</v>
@@ -61671,7 +61677,7 @@
         <v>6</v>
       </c>
       <c r="D2641" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2641" t="s" s="3">
         <v>5240</v>
@@ -61688,7 +61694,7 @@
         <v>6</v>
       </c>
       <c r="D2642" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2642" t="s" s="3">
         <v>5242</v>
@@ -61705,7 +61711,7 @@
         <v>6</v>
       </c>
       <c r="D2643" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2643" t="s" s="3">
         <v>5244</v>
@@ -61722,7 +61728,7 @@
         <v>6</v>
       </c>
       <c r="D2644" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2644" t="s" s="3">
         <v>5246</v>
@@ -61739,7 +61745,7 @@
         <v>6</v>
       </c>
       <c r="D2645" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2645" t="s" s="3">
         <v>5248</v>
@@ -61756,7 +61762,7 @@
         <v>6</v>
       </c>
       <c r="D2646" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2646" t="s" s="3">
         <v>5250</v>
@@ -61773,7 +61779,7 @@
         <v>6</v>
       </c>
       <c r="D2647" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2647" t="s" s="3">
         <v>5252</v>
@@ -61790,7 +61796,7 @@
         <v>6</v>
       </c>
       <c r="D2648" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2648" t="s" s="3">
         <v>5254</v>
@@ -61807,7 +61813,7 @@
         <v>6</v>
       </c>
       <c r="D2649" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2649" t="s" s="3">
         <v>5256</v>
@@ -61824,7 +61830,7 @@
         <v>6</v>
       </c>
       <c r="D2650" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2650" t="s" s="3">
         <v>5258</v>
@@ -61841,7 +61847,7 @@
         <v>6</v>
       </c>
       <c r="D2651" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2651" t="s" s="3">
         <v>5260</v>
@@ -61858,7 +61864,7 @@
         <v>6</v>
       </c>
       <c r="D2652" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2652" t="s" s="3">
         <v>5262</v>
@@ -61875,7 +61881,7 @@
         <v>6</v>
       </c>
       <c r="D2653" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2653" t="s" s="3">
         <v>5264</v>
@@ -61892,7 +61898,7 @@
         <v>6</v>
       </c>
       <c r="D2654" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2654" t="s" s="3">
         <v>5266</v>
@@ -61909,7 +61915,7 @@
         <v>6</v>
       </c>
       <c r="D2655" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2655" t="s" s="3">
         <v>5268</v>
@@ -61926,7 +61932,7 @@
         <v>6</v>
       </c>
       <c r="D2656" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2656" t="s" s="3">
         <v>5270</v>
@@ -61943,7 +61949,7 @@
         <v>6</v>
       </c>
       <c r="D2657" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2657" t="s" s="3">
         <v>5272</v>
@@ -61960,7 +61966,7 @@
         <v>6</v>
       </c>
       <c r="D2658" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2658" t="s" s="3">
         <v>5274</v>
@@ -61977,7 +61983,7 @@
         <v>6</v>
       </c>
       <c r="D2659" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2659" t="s" s="3">
         <v>5276</v>
@@ -61994,7 +62000,7 @@
         <v>6</v>
       </c>
       <c r="D2660" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2660" t="s" s="3">
         <v>5278</v>
@@ -62011,7 +62017,7 @@
         <v>6</v>
       </c>
       <c r="D2661" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2661" t="s" s="3">
         <v>5280</v>
@@ -62028,7 +62034,7 @@
         <v>6</v>
       </c>
       <c r="D2662" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2662" t="s" s="3">
         <v>5282</v>
@@ -62045,7 +62051,7 @@
         <v>6</v>
       </c>
       <c r="D2663" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2663" t="s" s="3">
         <v>5284</v>
@@ -62062,7 +62068,7 @@
         <v>6</v>
       </c>
       <c r="D2664" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2664" t="s" s="3">
         <v>5286</v>
@@ -62079,7 +62085,7 @@
         <v>6</v>
       </c>
       <c r="D2665" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2665" t="s" s="3">
         <v>5288</v>
@@ -62096,7 +62102,7 @@
         <v>6</v>
       </c>
       <c r="D2666" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2666" t="s" s="3">
         <v>5290</v>
@@ -62113,7 +62119,7 @@
         <v>6</v>
       </c>
       <c r="D2667" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2667" t="s" s="3">
         <v>5292</v>
@@ -62130,7 +62136,7 @@
         <v>6</v>
       </c>
       <c r="D2668" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2668" t="s" s="3">
         <v>5294</v>
@@ -62147,7 +62153,7 @@
         <v>6</v>
       </c>
       <c r="D2669" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2669" t="s" s="3">
         <v>5296</v>
@@ -62164,7 +62170,7 @@
         <v>6</v>
       </c>
       <c r="D2670" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2670" t="s" s="3">
         <v>5298</v>
@@ -62181,7 +62187,7 @@
         <v>6</v>
       </c>
       <c r="D2671" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2671" t="s" s="3">
         <v>5300</v>
@@ -62198,7 +62204,7 @@
         <v>6</v>
       </c>
       <c r="D2672" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2672" t="s" s="3">
         <v>5302</v>
@@ -62215,7 +62221,7 @@
         <v>6</v>
       </c>
       <c r="D2673" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2673" t="s" s="3">
         <v>5304</v>
@@ -62226,16 +62232,16 @@
         <v>2673.0</v>
       </c>
       <c r="B2674" t="s" s="3">
-        <v>3439</v>
+        <v>5305</v>
       </c>
       <c r="C2674" t="s" s="2">
         <v>6</v>
       </c>
       <c r="D2674" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2674" t="s" s="3">
-        <v>5305</v>
+        <v>5306</v>
       </c>
     </row>
     <row r="2675" ht="36.0" customHeight="true">
@@ -62243,13 +62249,13 @@
         <v>2674.0</v>
       </c>
       <c r="B2675" t="s" s="3">
-        <v>5306</v>
+        <v>3439</v>
       </c>
       <c r="C2675" t="s" s="2">
         <v>6</v>
       </c>
       <c r="D2675" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2675" t="s" s="3">
         <v>5307</v>
@@ -62266,7 +62272,7 @@
         <v>6</v>
       </c>
       <c r="D2676" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2676" t="s" s="3">
         <v>5309</v>
@@ -62283,10 +62289,10 @@
         <v>6</v>
       </c>
       <c r="D2677" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2677" t="s" s="3">
-        <v>5152</v>
+        <v>5311</v>
       </c>
     </row>
     <row r="2678" ht="36.0" customHeight="true">
@@ -62294,16 +62300,16 @@
         <v>2677.0</v>
       </c>
       <c r="B2678" t="s" s="3">
-        <v>5311</v>
+        <v>5312</v>
       </c>
       <c r="C2678" t="s" s="2">
         <v>6</v>
       </c>
       <c r="D2678" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2678" t="s" s="3">
-        <v>5312</v>
+        <v>5154</v>
       </c>
     </row>
     <row r="2679" ht="36.0" customHeight="true">
@@ -62317,7 +62323,7 @@
         <v>6</v>
       </c>
       <c r="D2679" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2679" t="s" s="3">
         <v>5314</v>
@@ -62334,7 +62340,7 @@
         <v>6</v>
       </c>
       <c r="D2680" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2680" t="s" s="3">
         <v>5316</v>
@@ -62351,7 +62357,7 @@
         <v>6</v>
       </c>
       <c r="D2681" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2681" t="s" s="3">
         <v>5318</v>
@@ -62368,7 +62374,7 @@
         <v>6</v>
       </c>
       <c r="D2682" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2682" t="s" s="3">
         <v>5320</v>
@@ -62385,7 +62391,7 @@
         <v>6</v>
       </c>
       <c r="D2683" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2683" t="s" s="3">
         <v>5322</v>
@@ -62402,7 +62408,7 @@
         <v>6</v>
       </c>
       <c r="D2684" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2684" t="s" s="3">
         <v>5324</v>
@@ -62416,10 +62422,10 @@
         <v>5325</v>
       </c>
       <c r="C2685" t="s" s="2">
-        <v>792</v>
+        <v>6</v>
       </c>
       <c r="D2685" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2685" t="s" s="3">
         <v>5326</v>
@@ -62436,7 +62442,7 @@
         <v>792</v>
       </c>
       <c r="D2686" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2686" t="s" s="3">
         <v>5328</v>
@@ -62453,7 +62459,7 @@
         <v>792</v>
       </c>
       <c r="D2687" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2687" t="s" s="3">
         <v>5330</v>
@@ -62470,7 +62476,7 @@
         <v>792</v>
       </c>
       <c r="D2688" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2688" t="s" s="3">
         <v>5332</v>
@@ -62487,7 +62493,7 @@
         <v>792</v>
       </c>
       <c r="D2689" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2689" t="s" s="3">
         <v>5334</v>
@@ -62504,7 +62510,7 @@
         <v>792</v>
       </c>
       <c r="D2690" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2690" t="s" s="3">
         <v>5336</v>
@@ -62521,7 +62527,7 @@
         <v>792</v>
       </c>
       <c r="D2691" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2691" t="s" s="3">
         <v>5338</v>
@@ -62538,7 +62544,7 @@
         <v>792</v>
       </c>
       <c r="D2692" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2692" t="s" s="3">
         <v>5340</v>
@@ -62555,7 +62561,7 @@
         <v>792</v>
       </c>
       <c r="D2693" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2693" t="s" s="3">
         <v>5342</v>
@@ -62572,7 +62578,7 @@
         <v>792</v>
       </c>
       <c r="D2694" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2694" t="s" s="3">
         <v>5344</v>
@@ -62589,7 +62595,7 @@
         <v>792</v>
       </c>
       <c r="D2695" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2695" t="s" s="3">
         <v>5346</v>
@@ -62606,7 +62612,7 @@
         <v>792</v>
       </c>
       <c r="D2696" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2696" t="s" s="3">
         <v>5348</v>
@@ -62623,7 +62629,7 @@
         <v>792</v>
       </c>
       <c r="D2697" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2697" t="s" s="3">
         <v>5350</v>
@@ -62640,7 +62646,7 @@
         <v>792</v>
       </c>
       <c r="D2698" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2698" t="s" s="3">
         <v>5352</v>
@@ -62657,7 +62663,7 @@
         <v>792</v>
       </c>
       <c r="D2699" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2699" t="s" s="3">
         <v>5354</v>
@@ -62674,7 +62680,7 @@
         <v>792</v>
       </c>
       <c r="D2700" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2700" t="s" s="3">
         <v>5356</v>
@@ -62691,7 +62697,7 @@
         <v>792</v>
       </c>
       <c r="D2701" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2701" t="s" s="3">
         <v>5358</v>
@@ -62708,7 +62714,7 @@
         <v>792</v>
       </c>
       <c r="D2702" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2702" t="s" s="3">
         <v>5360</v>
@@ -62725,7 +62731,7 @@
         <v>792</v>
       </c>
       <c r="D2703" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2703" t="s" s="3">
         <v>5362</v>
@@ -62742,7 +62748,7 @@
         <v>792</v>
       </c>
       <c r="D2704" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2704" t="s" s="3">
         <v>5364</v>
@@ -62759,7 +62765,7 @@
         <v>792</v>
       </c>
       <c r="D2705" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2705" t="s" s="3">
         <v>5366</v>
@@ -62776,7 +62782,7 @@
         <v>792</v>
       </c>
       <c r="D2706" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2706" t="s" s="3">
         <v>5368</v>
@@ -62793,7 +62799,7 @@
         <v>792</v>
       </c>
       <c r="D2707" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2707" t="s" s="3">
         <v>5370</v>
@@ -62810,7 +62816,7 @@
         <v>792</v>
       </c>
       <c r="D2708" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2708" t="s" s="3">
         <v>5372</v>
@@ -62827,7 +62833,7 @@
         <v>792</v>
       </c>
       <c r="D2709" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2709" t="s" s="3">
         <v>5374</v>
@@ -62844,7 +62850,7 @@
         <v>792</v>
       </c>
       <c r="D2710" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2710" t="s" s="3">
         <v>5376</v>
@@ -62861,7 +62867,7 @@
         <v>792</v>
       </c>
       <c r="D2711" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2711" t="s" s="3">
         <v>5378</v>
@@ -62878,7 +62884,7 @@
         <v>792</v>
       </c>
       <c r="D2712" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2712" t="s" s="3">
         <v>5380</v>
@@ -62895,7 +62901,7 @@
         <v>792</v>
       </c>
       <c r="D2713" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2713" t="s" s="3">
         <v>5382</v>
@@ -62912,7 +62918,7 @@
         <v>792</v>
       </c>
       <c r="D2714" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2714" t="s" s="3">
         <v>5384</v>
@@ -62929,7 +62935,7 @@
         <v>792</v>
       </c>
       <c r="D2715" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2715" t="s" s="3">
         <v>5386</v>
@@ -62946,7 +62952,7 @@
         <v>792</v>
       </c>
       <c r="D2716" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2716" t="s" s="3">
         <v>5388</v>
@@ -62963,7 +62969,7 @@
         <v>792</v>
       </c>
       <c r="D2717" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2717" t="s" s="3">
         <v>5390</v>
@@ -62980,7 +62986,7 @@
         <v>792</v>
       </c>
       <c r="D2718" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2718" t="s" s="3">
         <v>5392</v>
@@ -62997,7 +63003,7 @@
         <v>792</v>
       </c>
       <c r="D2719" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2719" t="s" s="3">
         <v>5394</v>
@@ -63014,7 +63020,7 @@
         <v>792</v>
       </c>
       <c r="D2720" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2720" t="s" s="3">
         <v>5396</v>
@@ -63031,7 +63037,7 @@
         <v>792</v>
       </c>
       <c r="D2721" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2721" t="s" s="3">
         <v>5398</v>
@@ -63048,7 +63054,7 @@
         <v>792</v>
       </c>
       <c r="D2722" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2722" t="s" s="3">
         <v>5400</v>
@@ -63065,7 +63071,7 @@
         <v>792</v>
       </c>
       <c r="D2723" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2723" t="s" s="3">
         <v>5402</v>
@@ -63082,7 +63088,7 @@
         <v>792</v>
       </c>
       <c r="D2724" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2724" t="s" s="3">
         <v>5404</v>
@@ -63099,7 +63105,7 @@
         <v>792</v>
       </c>
       <c r="D2725" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2725" t="s" s="3">
         <v>5406</v>
@@ -63116,7 +63122,7 @@
         <v>792</v>
       </c>
       <c r="D2726" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2726" t="s" s="3">
         <v>5408</v>
@@ -63133,7 +63139,7 @@
         <v>792</v>
       </c>
       <c r="D2727" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2727" t="s" s="3">
         <v>5410</v>
@@ -63150,7 +63156,7 @@
         <v>792</v>
       </c>
       <c r="D2728" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2728" t="s" s="3">
         <v>5412</v>
@@ -63167,7 +63173,7 @@
         <v>792</v>
       </c>
       <c r="D2729" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2729" t="s" s="3">
         <v>5414</v>
@@ -63184,10 +63190,10 @@
         <v>792</v>
       </c>
       <c r="D2730" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2730" t="s" s="3">
-        <v>5088</v>
+        <v>5416</v>
       </c>
     </row>
     <row r="2731" ht="36.0" customHeight="true">
@@ -63195,16 +63201,16 @@
         <v>2730.0</v>
       </c>
       <c r="B2731" t="s" s="3">
-        <v>5416</v>
+        <v>5417</v>
       </c>
       <c r="C2731" t="s" s="2">
         <v>792</v>
       </c>
       <c r="D2731" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2731" t="s" s="3">
-        <v>5417</v>
+        <v>5090</v>
       </c>
     </row>
     <row r="2732" ht="36.0" customHeight="true">
@@ -63218,7 +63224,7 @@
         <v>792</v>
       </c>
       <c r="D2732" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2732" t="s" s="3">
         <v>5419</v>
@@ -63235,7 +63241,7 @@
         <v>792</v>
       </c>
       <c r="D2733" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2733" t="s" s="3">
         <v>5421</v>
@@ -63252,7 +63258,7 @@
         <v>792</v>
       </c>
       <c r="D2734" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2734" t="s" s="3">
         <v>5423</v>
@@ -63269,7 +63275,7 @@
         <v>792</v>
       </c>
       <c r="D2735" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2735" t="s" s="3">
         <v>5425</v>
@@ -63286,7 +63292,7 @@
         <v>792</v>
       </c>
       <c r="D2736" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2736" t="s" s="3">
         <v>5427</v>
@@ -63303,7 +63309,7 @@
         <v>792</v>
       </c>
       <c r="D2737" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2737" t="s" s="3">
         <v>5429</v>
@@ -63317,10 +63323,10 @@
         <v>5430</v>
       </c>
       <c r="C2738" t="s" s="2">
-        <v>1011</v>
+        <v>792</v>
       </c>
       <c r="D2738" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2738" t="s" s="3">
         <v>5431</v>
@@ -63337,7 +63343,7 @@
         <v>1011</v>
       </c>
       <c r="D2739" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2739" t="s" s="3">
         <v>5433</v>
@@ -63348,16 +63354,16 @@
         <v>2739.0</v>
       </c>
       <c r="B2740" t="s" s="3">
-        <v>5411</v>
+        <v>5434</v>
       </c>
       <c r="C2740" t="s" s="2">
         <v>1011</v>
       </c>
       <c r="D2740" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2740" t="s" s="3">
-        <v>5434</v>
+        <v>5435</v>
       </c>
     </row>
     <row r="2741" ht="36.0" customHeight="true">
@@ -63365,13 +63371,13 @@
         <v>2740.0</v>
       </c>
       <c r="B2741" t="s" s="3">
-        <v>5435</v>
+        <v>5413</v>
       </c>
       <c r="C2741" t="s" s="2">
         <v>1011</v>
       </c>
       <c r="D2741" t="s" s="2">
-        <v>5031</v>
+        <v>5033</v>
       </c>
       <c r="E2741" t="s" s="3">
         <v>5436</v>
@@ -63385,13 +63391,13 @@
         <v>5437</v>
       </c>
       <c r="C2742" t="s" s="2">
-        <v>6</v>
+        <v>1011</v>
       </c>
       <c r="D2742" t="s" s="2">
+        <v>5033</v>
+      </c>
+      <c r="E2742" t="s" s="3">
         <v>5438</v>
-      </c>
-      <c r="E2742" t="s" s="3">
-        <v>5439</v>
       </c>
     </row>
     <row r="2743" ht="36.0" customHeight="true">
@@ -63399,13 +63405,13 @@
         <v>2742.0</v>
       </c>
       <c r="B2743" t="s" s="3">
+        <v>5439</v>
+      </c>
+      <c r="C2743" t="s" s="2">
+        <v>6</v>
+      </c>
+      <c r="D2743" t="s" s="2">
         <v>5440</v>
-      </c>
-      <c r="C2743" t="s" s="2">
-        <v>6</v>
-      </c>
-      <c r="D2743" t="s" s="2">
-        <v>5438</v>
       </c>
       <c r="E2743" t="s" s="3">
         <v>5441</v>
@@ -63422,7 +63428,7 @@
         <v>6</v>
       </c>
       <c r="D2744" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2744" t="s" s="3">
         <v>5443</v>
@@ -63439,7 +63445,7 @@
         <v>6</v>
       </c>
       <c r="D2745" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2745" t="s" s="3">
         <v>5445</v>
@@ -63456,7 +63462,7 @@
         <v>6</v>
       </c>
       <c r="D2746" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2746" t="s" s="3">
         <v>5447</v>
@@ -63473,7 +63479,7 @@
         <v>6</v>
       </c>
       <c r="D2747" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2747" t="s" s="3">
         <v>5449</v>
@@ -63490,7 +63496,7 @@
         <v>6</v>
       </c>
       <c r="D2748" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2748" t="s" s="3">
         <v>5451</v>
@@ -63507,7 +63513,7 @@
         <v>6</v>
       </c>
       <c r="D2749" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2749" t="s" s="3">
         <v>5453</v>
@@ -63524,7 +63530,7 @@
         <v>6</v>
       </c>
       <c r="D2750" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2750" t="s" s="3">
         <v>5455</v>
@@ -63541,7 +63547,7 @@
         <v>6</v>
       </c>
       <c r="D2751" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2751" t="s" s="3">
         <v>5457</v>
@@ -63558,7 +63564,7 @@
         <v>6</v>
       </c>
       <c r="D2752" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2752" t="s" s="3">
         <v>5459</v>
@@ -63575,7 +63581,7 @@
         <v>6</v>
       </c>
       <c r="D2753" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2753" t="s" s="3">
         <v>5461</v>
@@ -63592,7 +63598,7 @@
         <v>6</v>
       </c>
       <c r="D2754" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2754" t="s" s="3">
         <v>5463</v>
@@ -63609,7 +63615,7 @@
         <v>6</v>
       </c>
       <c r="D2755" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2755" t="s" s="3">
         <v>5465</v>
@@ -63626,7 +63632,7 @@
         <v>6</v>
       </c>
       <c r="D2756" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2756" t="s" s="3">
         <v>5467</v>
@@ -63643,7 +63649,7 @@
         <v>6</v>
       </c>
       <c r="D2757" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2757" t="s" s="3">
         <v>5469</v>
@@ -63660,7 +63666,7 @@
         <v>6</v>
       </c>
       <c r="D2758" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2758" t="s" s="3">
         <v>5471</v>
@@ -63677,7 +63683,7 @@
         <v>6</v>
       </c>
       <c r="D2759" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2759" t="s" s="3">
         <v>5473</v>
@@ -63694,7 +63700,7 @@
         <v>6</v>
       </c>
       <c r="D2760" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2760" t="s" s="3">
         <v>5475</v>
@@ -63711,7 +63717,7 @@
         <v>6</v>
       </c>
       <c r="D2761" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2761" t="s" s="3">
         <v>5477</v>
@@ -63728,7 +63734,7 @@
         <v>6</v>
       </c>
       <c r="D2762" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2762" t="s" s="3">
         <v>5479</v>
@@ -63745,7 +63751,7 @@
         <v>6</v>
       </c>
       <c r="D2763" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2763" t="s" s="3">
         <v>5481</v>
@@ -63762,7 +63768,7 @@
         <v>6</v>
       </c>
       <c r="D2764" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2764" t="s" s="3">
         <v>5483</v>
@@ -63779,7 +63785,7 @@
         <v>6</v>
       </c>
       <c r="D2765" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2765" t="s" s="3">
         <v>5485</v>
@@ -63796,7 +63802,7 @@
         <v>6</v>
       </c>
       <c r="D2766" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2766" t="s" s="3">
         <v>5487</v>
@@ -63813,7 +63819,7 @@
         <v>6</v>
       </c>
       <c r="D2767" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2767" t="s" s="3">
         <v>5489</v>
@@ -63830,7 +63836,7 @@
         <v>6</v>
       </c>
       <c r="D2768" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2768" t="s" s="3">
         <v>5491</v>
@@ -63847,7 +63853,7 @@
         <v>6</v>
       </c>
       <c r="D2769" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2769" t="s" s="3">
         <v>5493</v>
@@ -63864,7 +63870,7 @@
         <v>6</v>
       </c>
       <c r="D2770" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2770" t="s" s="3">
         <v>5495</v>
@@ -63881,7 +63887,7 @@
         <v>6</v>
       </c>
       <c r="D2771" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2771" t="s" s="3">
         <v>5497</v>
@@ -63898,7 +63904,7 @@
         <v>6</v>
       </c>
       <c r="D2772" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2772" t="s" s="3">
         <v>5499</v>
@@ -63915,7 +63921,7 @@
         <v>6</v>
       </c>
       <c r="D2773" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2773" t="s" s="3">
         <v>5501</v>
@@ -63932,7 +63938,7 @@
         <v>6</v>
       </c>
       <c r="D2774" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2774" t="s" s="3">
         <v>5503</v>
@@ -63949,7 +63955,7 @@
         <v>6</v>
       </c>
       <c r="D2775" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2775" t="s" s="3">
         <v>5505</v>
@@ -63966,7 +63972,7 @@
         <v>6</v>
       </c>
       <c r="D2776" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2776" t="s" s="3">
         <v>5507</v>
@@ -63983,7 +63989,7 @@
         <v>6</v>
       </c>
       <c r="D2777" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2777" t="s" s="3">
         <v>5509</v>
@@ -64000,7 +64006,7 @@
         <v>6</v>
       </c>
       <c r="D2778" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2778" t="s" s="3">
         <v>5511</v>
@@ -64014,13 +64020,13 @@
         <v>5512</v>
       </c>
       <c r="C2779" t="s" s="2">
-        <v>792</v>
+        <v>6</v>
       </c>
       <c r="D2779" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2779" t="s" s="3">
-        <v>5485</v>
+        <v>5513</v>
       </c>
     </row>
     <row r="2780" ht="36.0" customHeight="true">
@@ -64028,16 +64034,16 @@
         <v>2779.0</v>
       </c>
       <c r="B2780" t="s" s="3">
-        <v>5513</v>
+        <v>5514</v>
       </c>
       <c r="C2780" t="s" s="2">
         <v>792</v>
       </c>
       <c r="D2780" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2780" t="s" s="3">
-        <v>5514</v>
+        <v>5487</v>
       </c>
     </row>
     <row r="2781" ht="36.0" customHeight="true">
@@ -64051,7 +64057,7 @@
         <v>792</v>
       </c>
       <c r="D2781" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2781" t="s" s="3">
         <v>5516</v>
@@ -64068,7 +64074,7 @@
         <v>792</v>
       </c>
       <c r="D2782" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2782" t="s" s="3">
         <v>5518</v>
@@ -64085,7 +64091,7 @@
         <v>792</v>
       </c>
       <c r="D2783" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2783" t="s" s="3">
         <v>5520</v>
@@ -64102,7 +64108,7 @@
         <v>792</v>
       </c>
       <c r="D2784" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2784" t="s" s="3">
         <v>5522</v>
@@ -64113,16 +64119,16 @@
         <v>2784.0</v>
       </c>
       <c r="B2785" t="s" s="3">
-        <v>5446</v>
+        <v>5523</v>
       </c>
       <c r="C2785" t="s" s="2">
         <v>792</v>
       </c>
       <c r="D2785" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2785" t="s" s="3">
-        <v>5523</v>
+        <v>5524</v>
       </c>
     </row>
     <row r="2786" ht="36.0" customHeight="true">
@@ -64130,13 +64136,13 @@
         <v>2785.0</v>
       </c>
       <c r="B2786" t="s" s="3">
-        <v>5524</v>
+        <v>5448</v>
       </c>
       <c r="C2786" t="s" s="2">
         <v>792</v>
       </c>
       <c r="D2786" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2786" t="s" s="3">
         <v>5525</v>
@@ -64153,7 +64159,7 @@
         <v>792</v>
       </c>
       <c r="D2787" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2787" t="s" s="3">
         <v>5527</v>
@@ -64170,7 +64176,7 @@
         <v>792</v>
       </c>
       <c r="D2788" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2788" t="s" s="3">
         <v>5529</v>
@@ -64187,7 +64193,7 @@
         <v>792</v>
       </c>
       <c r="D2789" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2789" t="s" s="3">
         <v>5531</v>
@@ -64204,7 +64210,7 @@
         <v>792</v>
       </c>
       <c r="D2790" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2790" t="s" s="3">
         <v>5533</v>
@@ -64221,7 +64227,7 @@
         <v>792</v>
       </c>
       <c r="D2791" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2791" t="s" s="3">
         <v>5535</v>
@@ -64238,7 +64244,7 @@
         <v>792</v>
       </c>
       <c r="D2792" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2792" t="s" s="3">
         <v>5537</v>
@@ -64255,7 +64261,7 @@
         <v>792</v>
       </c>
       <c r="D2793" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2793" t="s" s="3">
         <v>5539</v>
@@ -64272,7 +64278,7 @@
         <v>792</v>
       </c>
       <c r="D2794" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2794" t="s" s="3">
         <v>5541</v>
@@ -64289,7 +64295,7 @@
         <v>792</v>
       </c>
       <c r="D2795" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2795" t="s" s="3">
         <v>5543</v>
@@ -64306,7 +64312,7 @@
         <v>792</v>
       </c>
       <c r="D2796" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2796" t="s" s="3">
         <v>5545</v>
@@ -64323,7 +64329,7 @@
         <v>792</v>
       </c>
       <c r="D2797" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2797" t="s" s="3">
         <v>5547</v>
@@ -64340,7 +64346,7 @@
         <v>792</v>
       </c>
       <c r="D2798" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2798" t="s" s="3">
         <v>5549</v>
@@ -64357,7 +64363,7 @@
         <v>792</v>
       </c>
       <c r="D2799" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2799" t="s" s="3">
         <v>5551</v>
@@ -64374,7 +64380,7 @@
         <v>792</v>
       </c>
       <c r="D2800" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2800" t="s" s="3">
         <v>5553</v>
@@ -64391,10 +64397,27 @@
         <v>792</v>
       </c>
       <c r="D2801" t="s" s="2">
-        <v>5438</v>
+        <v>5440</v>
       </c>
       <c r="E2801" t="s" s="3">
         <v>5555</v>
+      </c>
+    </row>
+    <row r="2802" ht="36.0" customHeight="true">
+      <c r="A2802" t="n" s="2">
+        <v>2801.0</v>
+      </c>
+      <c r="B2802" t="s" s="3">
+        <v>5556</v>
+      </c>
+      <c r="C2802" t="s" s="2">
+        <v>792</v>
+      </c>
+      <c r="D2802" t="s" s="2">
+        <v>5440</v>
+      </c>
+      <c r="E2802" t="s" s="3">
+        <v>5557</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
로봇 자동 갱신: 2026-10-25
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -6374,10 +6374,10 @@
     <t>그리너리 바스켓</t>
   </si>
   <si>
+    <t>인천광역시 영종구 백운로 510(2동 1,2층 운북동)</t>
+  </si>
+  <si>
     <t>인천광역시 영종구 백운로 510(1동 지1층 운북동)</t>
-  </si>
-  <si>
-    <t>인천광역시 영종구 백운로 510(2동 1,2층 운북동)</t>
   </si>
   <si>
     <t>까페마인</t>

</xml_diff>